<commit_message>
PostgreSQL production database setup
</commit_message>
<xml_diff>
--- a/Har_Ghar_Solar_Leads.xlsx
+++ b/Har_Ghar_Solar_Leads.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$I$3</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -415,19 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -437,12 +424,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Customer_Name</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -452,7 +439,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Electricity_Bill</t>
+          <t>Bill</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -462,17 +449,17 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Follow_Notes</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Follow_Date</t>
+          <t>Follow Date</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Lead_Date</t>
+          <t>Created</t>
         </is>
       </c>
     </row>
@@ -482,22 +469,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SUMIT GOSWAMI</t>
+          <t>KAKA1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>08077181038</t>
+          <t>9876543210</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Chanduasi</t>
+          <t>Sambhal</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Above ₹5000</t>
+          <t>₹3000 - ₹5000</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -505,59 +492,23 @@
           <t>New</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Thanks</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>10-07-2026 01:27 PM</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>SUMIT GOSWAMI</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>08077181038</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Chanduasi</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Above ₹5000</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Installed</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>fdhdfdfj</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>2026-07-09</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>10-07-2026 01:28 PM</t>
+          <t>2026-07-10</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>